<commit_message>
Update .gitignore, add validation scripts and Excel files for piece availability
</commit_message>
<xml_diff>
--- a/pecas-por-rota/tabela_lojas_rotas.xlsx
+++ b/pecas-por-rota/tabela_lojas_rotas.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C77"/>
+  <dimension ref="A1:E85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -429,7 +429,17 @@
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Unidade de Negócio</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Max Peças</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Qtd. Ruas</t>
         </is>
       </c>
     </row>
@@ -446,8 +456,14 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -458,13 +474,19 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>TP PF 87</t>
+          <t>504-87</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -480,8 +502,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>5500</v>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -497,8 +525,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -509,13 +543,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TP PF 6</t>
+          <t>504-6</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -526,13 +566,19 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>TP PF 5J</t>
+          <t>504-5J</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -543,13 +589,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TP PF 6</t>
+          <t>504-6</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -560,13 +612,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TP PF 88</t>
+          <t>504-88</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -577,13 +635,19 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TP PF 88</t>
+          <t>504-88</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -599,8 +663,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -616,8 +686,14 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -633,8 +709,14 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -645,13 +727,19 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>TP PF 5J</t>
+          <t>504-5J</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Camicado</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -662,13 +750,19 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
+          <t>504-5R</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Camicado</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -679,13 +773,19 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TP PF 6</t>
+          <t>504-6</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Camicado</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -696,13 +796,19 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
+          <t>504-5R</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Camicado</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1000</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -713,13 +819,19 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
+          <t>504-5R</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -730,13 +842,19 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
+          <t>504-5R</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="20">
@@ -747,13 +865,19 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>TP PF 84B</t>
+          <t>504-84B</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -764,13 +888,19 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
+          <t>504-5R</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22">
@@ -786,327 +916,503 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>40057</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr"/>
+          <t>40051</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>504-87</t>
+        </is>
+      </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>40078</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr"/>
+          <t>40057</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>TP PF 86</t>
+        </is>
+      </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>40080</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr"/>
+          <t>40078</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>504-84B</t>
+        </is>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>40089</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr"/>
+          <t>40080</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>504-84B</t>
+        </is>
+      </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>40105</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr"/>
+          <t>40089</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>TP PF 86</t>
+        </is>
+      </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E27" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>40119</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr"/>
+          <t>40091</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>504-5R</t>
+        </is>
+      </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E28" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>40143</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr"/>
+          <t>40105</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>504-88</t>
+        </is>
+      </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>40158</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr"/>
+          <t>40106</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>504-6</t>
+        </is>
+      </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E30" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>40160</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr"/>
+          <t>40108</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>504-87</t>
+        </is>
+      </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>40163</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr"/>
+          <t>40111</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>504-5R</t>
+        </is>
+      </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E32" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>40179</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr"/>
+          <t>40119</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>TP PF 89</t>
+        </is>
+      </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>PENDENTE - preencher rota manualmente</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E33" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>40121</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>TP PF 89</t>
+          <t>504-5J</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E34" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>427</t>
+          <t>40139</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>TP PF 87</t>
+          <t>504-6</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E35" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>430</t>
+          <t>40143</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
+          <t>TP PF 85</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E36" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>448</t>
+          <t>40158</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>TP PF 84A</t>
+          <t>TP PF 85</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>455</t>
+          <t>40160</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>TP PF 5J</t>
+          <t>TP PF 86</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E38" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>476</t>
+          <t>40163</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TP PF 84B</t>
+          <t>TP PF 85</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>478</t>
+          <t>40179</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TP PF 84B</t>
+          <t>504-88</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Youcom</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>502</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>TP PF 6</t>
+          <t>TP PF 89</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E41" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>509</t>
+          <t>427</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
+          <t>504-87</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>516</t>
+          <t>430</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TP PF 6</t>
+          <t>504-5R</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E43" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>533</t>
+          <t>448</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1116,133 +1422,181 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E44" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>535</t>
+          <t>455</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>TP PF 84A</t>
+          <t>504-5J</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>476</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>TP PF 85</t>
+          <t>504-84B</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>560</t>
+          <t>478</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>TP PF 6</t>
+          <t>504-84B</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1900</v>
+      </c>
+      <c r="E47" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>570</t>
+          <t>502</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TP PF 6</t>
+          <t>504-6</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E48" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>580</t>
+          <t>509</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>TP PF 85</t>
+          <t>504-5R</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>588</t>
+          <t>516</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TP PF 87</t>
+          <t>504-6</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>533</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TP PF 88</t>
+          <t>TP PF 84A</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>610</t>
+          <t>535</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1252,434 +1606,638 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>611</t>
+          <t>550</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
+          <t>TP PF 85</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>560</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TP PF 86</t>
+          <t>504-6</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>720</t>
+          <t>570</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>TP PF 84A</t>
+          <t>504-6</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Preenchida manualmente</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E55" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>73</t>
+          <t>580</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
+          <t>TP PF 85</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>76</t>
+          <t>588</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>TP PF 84B</t>
+          <t>504-87</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>2750</v>
+      </c>
+      <c r="E57" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>600</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>TP PF 5J</t>
+          <t>504-88</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>606</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>TP PF 86</t>
+          <t>504-5R</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E59" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>610</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>TP PF 89</t>
+          <t>TP PF 84A</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E60" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>AS720</t>
+          <t>611</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TP PF 87</t>
+          <t>504-5R</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>3000</v>
+      </c>
+      <c r="E61" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>YC051</t>
+          <t>68</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>TP PF 87</t>
+          <t>TP PF 86</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>7000</v>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>YC057</t>
+          <t>720</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>TP PF 86</t>
+          <t>504-87</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Ashua</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E63" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>YC089</t>
+          <t>73</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>TP PF 86</t>
+          <t>504-5R</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E64" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>YC091</t>
+          <t>76</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
+          <t>504-84B</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E65" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>YC105</t>
+          <t>77</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>TP PF 88</t>
+          <t>504-5J</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>YC106</t>
+          <t>83</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>TP PF 6</t>
+          <t>TP PF 86</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E67" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>YC108</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>TP PF 87</t>
+          <t>TP PF 89</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
+          <t>Renner</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>5000</v>
+      </c>
+      <c r="E68" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>YC111</t>
+          <t>AS720</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>TP PF 5R</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
-      </c>
+          <t>TP PF 87</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr"/>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>YC119</t>
+          <t>YC051</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>TP PF 89</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
-      </c>
+          <t>TP PF 87</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr"/>
+      <c r="D70" t="inlineStr"/>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>YC121</t>
+          <t>YC057</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>TP PF 5J</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
-      </c>
+          <t>TP PF 86</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr"/>
+      <c r="D71" t="inlineStr"/>
+      <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>YC139</t>
+          <t>YC089</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>TP PF 6</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
-      </c>
+          <t>TP PF 86</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>YC143</t>
+          <t>YC091</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>TP PF 85</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
-      </c>
+          <t>TP PF 5R</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr"/>
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>YC158</t>
+          <t>YC105</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>TP PF 85</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
-      </c>
+          <t>TP PF 88</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr"/>
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>YC160</t>
+          <t>YC106</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>TP PF 86</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
-      </c>
+          <t>TP PF 6</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>YC163</t>
+          <t>YC108</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>TP PF 85</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
-      </c>
+          <t>TP PF 87</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr"/>
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
+          <t>YC111</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>TP PF 5R</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr"/>
+      <c r="D77" t="inlineStr"/>
+      <c r="E77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>YC119</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>TP PF 89</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
+      <c r="D78" t="inlineStr"/>
+      <c r="E78" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>YC121</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>TP PF 5J</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr"/>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>YC139</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>TP PF 6</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr"/>
+      <c r="D80" t="inlineStr"/>
+      <c r="E80" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>YC143</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>TP PF 85</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr"/>
+      <c r="D81" t="inlineStr"/>
+      <c r="E81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>YC158</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>TP PF 85</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr"/>
+      <c r="D82" t="inlineStr"/>
+      <c r="E82" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>YC160</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>TP PF 86</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr"/>
+      <c r="D83" t="inlineStr"/>
+      <c r="E83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>YC163</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>TP PF 85</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr"/>
+      <c r="D84" t="inlineStr"/>
+      <c r="E84" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
           <t>YC179</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>TP PF 88</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Cadastrada automaticamente pela programação</t>
-        </is>
-      </c>
+      <c r="C85" t="inlineStr"/>
+      <c r="D85" t="inlineStr"/>
+      <c r="E85" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>